<commit_message>
Refresh roof price registry mappings
</commit_message>
<xml_diff>
--- a/output/price_registry_filled_v4.xlsx
+++ b/output/price_registry_filled_v4.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H194"/>
+  <dimension ref="A1:H195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -572,7 +572,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -5212,7 +5212,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -6101,7 +6101,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -6199,28 +6199,28 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Монтаж примыкания к вентшахтам</t>
+          <t>Монтаж примыкания кровли из ПВХ мембраны</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>мп</t>
         </is>
       </c>
       <c r="D186" t="n">
         <v>1</v>
       </c>
       <c r="E186" t="n">
-        <v>5000</v>
+        <v>700</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Источник: первый лист нового прайса, строка 36. Исходное кол-во: 1.0. price_code задан ручной картой normalize_elena_price_registry.py.</t>
+          <t>Добавлено 2026-08-02 по сверке эталонных смет: общее линейное примыкание кровли к парапетам/стенам/ВК считается в м.п.; отдельное примыкание к вентшахтам в шт остается optional legacy.</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Установка аэратора кровельного PVC, А75х375</t>
+          <t>Монтаж примыкания к вентшахтам</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -6249,33 +6249,33 @@
         <v>1</v>
       </c>
       <c r="E187" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Добавлено по ответу Елены 2026-07-30: 587 руб. — материал аэратора, работа отдельно 2500 руб./шт.</t>
+          <t>Источник: первый лист нового прайса, строка 36. Исходное кол-во: 1.0. price_code задан ручной картой normalize_elena_price_registry.py.</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>roof_pvc_aerator_75x375_installation_item</t>
+          <t>roof_vent_shaft_abutment_installation_item</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Schiedel</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Вентиляционный канал одноходовой VENT 20/25, 0.33 пм</t>
+          <t>Установка аэратора кровельного PVC, А75х375</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -6287,14 +6287,21 @@
         <v>1</v>
       </c>
       <c r="E188" t="n">
-        <v>268.4</v>
-      </c>
-      <c r="F188" s="2" t="n">
-        <v>46146</v>
+        <v>2500</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Вместимость в машину: h=330мм, габариты 200×250мм, вес 13кг, 63 шт на поддоне Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+          <t>Добавлено по ответу Елены 2026-07-30: 587 руб. — материал аэратора, работа отдельно 2500 руб./шт.</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>roof_pvc_aerator_75x375_installation_item</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6313,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Вентиляционный канал четырехходовой VENT 36/50, 0.33 пм</t>
+          <t>Вентиляционный канал одноходовой VENT 20/25, 0.33 пм</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -6318,14 +6325,14 @@
         <v>1</v>
       </c>
       <c r="E189" t="n">
-        <v>902.8</v>
+        <v>268.4</v>
       </c>
       <c r="F189" s="2" t="n">
         <v>46146</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Вместимость в машину: h=330мм, габариты 500×360мм, вес 38кг, 16 шт на поддоне Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+          <t>Вместимость в машину: h=330мм, габариты 200×250мм, вес 13кг, 63 шт на поддоне Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6344,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Вентиляционный канал одноходовой VENT 16/25-1X, 0.33 пм</t>
+          <t>Вентиляционный канал четырехходовой VENT 36/50, 0.33 пм</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -6349,14 +6356,14 @@
         <v>1</v>
       </c>
       <c r="E190" t="n">
-        <v>264</v>
+        <v>902.8</v>
       </c>
       <c r="F190" s="2" t="n">
         <v>46146</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+          <t>Вместимость в машину: h=330мм, габариты 500×360мм, вес 38кг, 16 шт на поддоне Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -6368,7 +6375,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Вентиляционный канал двухходовой VENT 16/50-2X, 0.33 пм</t>
+          <t>Вентиляционный канал одноходовой VENT 16/25-1X, 0.33 пм</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -6380,7 +6387,7 @@
         <v>1</v>
       </c>
       <c r="E191" t="n">
-        <v>672</v>
+        <v>264</v>
       </c>
       <c r="F191" s="2" t="n">
         <v>46146</v>
@@ -6399,7 +6406,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Вентиляционный канал двухходовой VENT 25/36, 0.33 пм</t>
+          <t>Вентиляционный канал двухходовой VENT 16/50-2X, 0.33 пм</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -6411,19 +6418,14 @@
         <v>1</v>
       </c>
       <c r="E192" t="n">
-        <v>512.4</v>
+        <v>672</v>
       </c>
       <c r="F192" s="2" t="n">
         <v>46146</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Вместимость в машину: h=330мм, габариты 250×360мм, вес 21кг, 36 шт на поддоне</t>
-        </is>
-      </c>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>schiedel_vent_channel_2x_36_25_item</t>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6437,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Вентиляционный канал трехходовой VENT 25/52, 0.33 пм</t>
+          <t>Вентиляционный канал двухходовой VENT 25/36, 0.33 пм</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -6447,57 +6449,93 @@
         <v>1</v>
       </c>
       <c r="E193" t="n">
-        <v>732</v>
+        <v>512.4</v>
       </c>
       <c r="F193" s="2" t="n">
         <v>46146</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Вместимость в машину: h=330мм, габариты 520×250мм, вес 31кг, 20 шт на поддоне</t>
+          <t>Вместимость в машину: h=330мм, габариты 250×360мм, вес 21кг, 36 шт на поддоне</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>schiedel_vent_channel_3x_52_25_item</t>
+          <t>schiedel_vent_channel_2x_36_25_item</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Schiedel</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Доставка вентканалов/ разгрузка в ручную на объекте</t>
+          <t>Вентиляционный канал трехходовой VENT 25/52, 0.33 пм</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>маш</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D194" t="n">
         <v>1</v>
       </c>
-      <c r="E194" t="inlineStr">
+      <c r="E194" t="n">
+        <v>732</v>
+      </c>
+      <c r="F194" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Вместимость в машину: h=330мм, габариты 520×250мм, вес 31кг, 20 шт на поддоне</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>schiedel_vent_channel_3x_52_25_item</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Доставка вентканалов/ разгрузка в ручную на объекте</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>1</v>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>2 500</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="G194" t="inlineStr">
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
         <is>
           <t>Источник: первый лист нового прайса, строка 42. Исходное кол-во: 1.0. price_code задан ручной картой normalize_elena_price_registry.py.</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr">
+      <c r="H195" t="inlineStr">
         <is>
           <t>schiedel_delivery_truck</t>
         </is>

</xml_diff>

<commit_message>
Fix walls/lintels pricing: split shared registry codes, correct section-specific rate
- cutoff_waterproofing_material_unit_price no longer shares its registry code
  with the work price (both resolved to the same 100 rub row) - added its own
  code, real value confirmed 250 rub/m2 on TRC and ARK.
- technical_supervision_amount no longer reuses a foundation_slab-labeled
  registry row (5000 rub) - added a dedicated code for this section, real TRC
  value is 10000 rub. First of the known ~16-row stale-placeholder queue closed
  with a confirmed per-section number.
</commit_message>
<xml_diff>
--- a/output/price_registry_filled_v4.xlsx
+++ b/output/price_registry_filled_v4.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H219"/>
+  <dimension ref="A1:H221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -512,7 +512,6 @@
           <t>Источник: первый лист нового прайса, строка 3. Исходное кол-во: 1. price_code не найден автоматически: нужно сопоставить вручную.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -546,7 +545,6 @@
           <t>Источник: первый лист нового прайса, строка 4. Исходное кол-во: 1. price_code не найден автоматически: нужно сопоставить вручную.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7510,7 +7508,82 @@
           <t>Источник: первый лист нового прайса, строка 42. Исходное кол-во: 1. price_code не найден автоматически: нужно сопоставить вручную.</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Гидроизоляция поверхности под первый ряд блоков, материал</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>1</v>
+      </c>
+      <c r="E220" t="n">
+        <v>250</v>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Добавлено 2026-08-09: material_unit_price ошибочно делил один registry_code с work_unit_price (cutoff_waterproofing_under_blocks_m2=100), из-за чего материал был занижен. Реальная цена материала подтверждена на ТРЦ и АРК (оба проекта: мат=250, работа=100, серый/реальный столбец) - см. отчёт 04_load_bearing_walls_lintels.md.</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>cutoff_waterproofing_material_m2</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Работы</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Технический надзор (стены/перемычки)</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>1</v>
+      </c>
+      <c r="E221" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Добавлено 2026-08-09: technical_supervision_amount ошибочно делил один registry_code (technical_supervision_fixed=5000) со строкой из раздела плиты фундамента. Реальная цена для раздела стен/перемычек подтверждена на ТРЦ (серый/реальный столбец) = 10000 - см. отчёт 04_load_bearing_walls_lintels.md.</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>technical_supervision_walls_lintels</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>